<commit_message>
feat(guia-churreria): Excel regenerados (gate_libros 8/8 verde) y documentos re-ensamblados tras la revisión — guía 95, BP 14, bonus 21, gates en verde
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/productos-digitales/guia-churreria/build/aceite-de-fritura-coste-y-cambio.xlsx
+++ b/scripts/productos-digitales/guia-churreria/build/aceite-de-fritura-coste-y-cambio.xlsx
@@ -3109,12 +3109,12 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="6">
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="D36:G36"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="D33:G33"/>
+    <mergeCell ref="D11:G11"/>
     <mergeCell ref="G18:G19"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="D40:G40"/>
-    <mergeCell ref="D11:G11"/>
   </mergeCells>
   <conditionalFormatting sqref="B21:D21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0" stopIfTrue="1">
@@ -3662,15 +3662,15 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="9">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A18:E18"/>
+    <mergeCell ref="F22:I22"/>
   </mergeCells>
   <conditionalFormatting sqref="H7:H14">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
@@ -4324,11 +4324,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="5">
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="B16:D16"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <conditionalFormatting sqref="B16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0" stopIfTrue="1">

</xml_diff>